<commit_message>
change RoCN to RoCStDv
</commit_message>
<xml_diff>
--- a/inst/extdata/ExampleDQO.xlsx
+++ b/inst/extdata/ExampleDQO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proj\AquaSensR\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{278A45A7-B7D6-4DB7-9C8F-AA9B0DCFD659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12204505-C047-4101-8CCE-F1256E212974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="252" windowWidth="21600" windowHeight="11232" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,9 +46,6 @@
     <t>Salinity_ppt</t>
   </si>
   <si>
-    <t>RoCN</t>
-  </si>
-  <si>
     <t>Flag</t>
   </si>
   <si>
@@ -77,6 +74,9 @@
   </si>
   <si>
     <t>Water_Temp_C</t>
+  </si>
+  <si>
+    <t>RoCStDv</t>
   </si>
 </sst>
 </file>
@@ -429,25 +429,25 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>13</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>14</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>15</v>
       </c>
-      <c r="G1" t="s">
-        <v>16</v>
-      </c>
       <c r="H1" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="I1" t="s">
         <v>1</v>
@@ -455,10 +455,10 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C2">
         <v>-0.5</v>
@@ -484,10 +484,10 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3">
         <v>-1</v>
@@ -505,10 +505,10 @@
         <v>0.01</v>
       </c>
       <c r="H3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -516,7 +516,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -545,7 +545,7 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5">
         <v>-1</v>
@@ -563,10 +563,10 @@
         <v>0.01</v>
       </c>
       <c r="H5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -574,7 +574,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -603,7 +603,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -621,10 +621,10 @@
         <v>0.01</v>
       </c>
       <c r="H7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -632,7 +632,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C8">
         <v>20</v>
@@ -661,7 +661,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C9">
         <v>10</v>
@@ -679,10 +679,10 @@
         <v>0.01</v>
       </c>
       <c r="H9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -690,7 +690,7 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C10">
         <v>20</v>
@@ -719,7 +719,7 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11">
         <v>10</v>
@@ -737,10 +737,10 @@
         <v>0.01</v>
       </c>
       <c r="H11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -748,7 +748,7 @@
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C12">
         <v>3</v>
@@ -777,7 +777,7 @@
         <v>7</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C13">
         <v>2</v>
@@ -795,10 +795,10 @@
         <v>0.01</v>
       </c>
       <c r="H13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -806,7 +806,7 @@
         <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C14">
         <v>4</v>
@@ -835,7 +835,7 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C15">
         <v>3</v>
@@ -853,10 +853,10 @@
         <v>0.01</v>
       </c>
       <c r="H15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
setup fail rate of change flags
</commit_message>
<xml_diff>
--- a/inst/extdata/ExampleDQO.xlsx
+++ b/inst/extdata/ExampleDQO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proj\AquaSensR\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12204505-C047-4101-8CCE-F1256E212974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE66F5CB-A5A1-4D3D-98D0-ACE4F84AF48E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="252" windowWidth="21600" windowHeight="11232" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="345" yWindow="555" windowWidth="15465" windowHeight="10665" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="19">
   <si>
     <t>Parameter</t>
   </si>
@@ -419,12 +419,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -453,7 +453,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -482,7 +482,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -504,14 +504,14 @@
       <c r="G3">
         <v>0.01</v>
       </c>
-      <c r="H3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -540,7 +540,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -569,7 +569,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -598,7 +598,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -627,7 +627,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -656,7 +656,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -685,7 +685,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -714,7 +714,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -743,7 +743,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -772,7 +772,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -801,7 +801,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -830,7 +830,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>4</v>
       </c>

</xml_diff>